<commit_message>
fix(control): correct drafting and animal patch integration
Reconstructed from original history (original Git tree retained).
Original checkpoint: cfbec172a6706fad3298d9b4e2b6bd118476b72e
</commit_message>
<xml_diff>
--- a/checker/Calculations.xlsx
+++ b/checker/Calculations.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Фотонозои\Обновленная сборка\Rimworld 1.6\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Фотонозои\Обновленная сборка\Rimworld 1.6\ZoologyFramework\checker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2FE57EB-E5F3-45D8-9E7D-34C6806B167D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38F50F34-3980-4B0C-A888-73D0ABFA5C69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="823" activeTab="2" xr2:uid="{6F854AE1-A176-497B-BE52-7B1B2A578D65}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="823" xr2:uid="{6F854AE1-A176-497B-BE52-7B1B2A578D65}"/>
   </bookViews>
   <sheets>
     <sheet name="Bite force" sheetId="17" r:id="rId1"/>
@@ -28,7 +28,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Teeth!$A$2:$D$221</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcMode="manual"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -459,7 +459,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1816" uniqueCount="649">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1904" uniqueCount="694">
   <si>
     <t>Struthio camelus</t>
   </si>
@@ -2888,6 +2888,141 @@
   <si>
     <t>https://www.pnas.org/doi/10.1073/pnas.0706086104</t>
   </si>
+  <si>
+    <t>Theropods</t>
+  </si>
+  <si>
+    <t>Sakamoto (2021) https://doi.org/10.1111/pala.12567</t>
+  </si>
+  <si>
+    <t>Carnotaurus sastrei</t>
+  </si>
+  <si>
+    <t>Dromaeosaurus albertensis</t>
+  </si>
+  <si>
+    <t>Majungasaurus crenatissimus</t>
+  </si>
+  <si>
+    <t>Tarbosaurus bataar</t>
+  </si>
+  <si>
+    <t>Sinraptor dongi</t>
+  </si>
+  <si>
+    <t>Herrerasaurus ischigualastensis</t>
+  </si>
+  <si>
+    <t>Coelophysis rhodesiensis</t>
+  </si>
+  <si>
+    <t>Daspletosaurus torosus</t>
+  </si>
+  <si>
+    <t>Gorgosaurus libratus</t>
+  </si>
+  <si>
+    <t>Lesothosaurus diagnosticus</t>
+  </si>
+  <si>
+    <t>corrected dry skull</t>
+  </si>
+  <si>
+    <t>Bates &amp; Falkingham (2012) and Sellers (2017) https://doi.org/10.1098/rsbl.2012.0056 https://peerj.com/articles/3420/</t>
+  </si>
+  <si>
+    <t>Sakamoto (2021) https://doi.org/10.1111/pala.12567 and https://www.reddit.com/r/Paleontology/comments/1kso8go/is_the_latest_mass_estimates_used_for_a_accurate</t>
+  </si>
+  <si>
+    <t>Acrocanthosaurus atokensis</t>
+  </si>
+  <si>
+    <t>Baryonyx walkeri</t>
+  </si>
+  <si>
+    <t>Carcharodontosaurus saharicus</t>
+  </si>
+  <si>
+    <t>Ceratosaurus nasicornis</t>
+  </si>
+  <si>
+    <t>Deinonychus antirrhopus</t>
+  </si>
+  <si>
+    <t>Gallimimus bullatus</t>
+  </si>
+  <si>
+    <t>Monolophosaurus jiangi</t>
+  </si>
+  <si>
+    <t>Spinosaurus aegyptiacus</t>
+  </si>
+  <si>
+    <t>Velociraptor mongoliensis</t>
+  </si>
+  <si>
+    <t>Yangchuanosaurus shangyouensis</t>
+  </si>
+  <si>
+    <t>Bates &amp; Falkingham (2012) https://doi.org/10.1098/rsbl.2012.0056 and https://www.deviantart.com/triceratopshorridus/journal/Predatory-Dinosaur-Size-Estimations-856766637?utm_source=chatgpt.com</t>
+  </si>
+  <si>
+    <t>Sakamoto (2021) https://doi.org/10.1111/pala.12567  and Sellers (2017) https://doi.org/10.1098/rsbl.2012.0056 https://peerj.com/articles/3420/</t>
+  </si>
+  <si>
+    <t>Sakamoto (2021) https://doi.org/10.1111/pala.12567 and https://www.miketaylor.org.uk/tmp/lovejoy/Erickson-et-al_04_tyrannosaurid-growth.pdf</t>
+  </si>
+  <si>
+    <t>Sakamoto (2021) https://doi.org/10.1111/pala.12567 and https://www.researchgate.net/publication/232687833_My_theropod_is_bigger_than_yoursor_not_Estimating_body_size_from_skull_length_in_theropods?utm_source=chatgpt.com</t>
+  </si>
+  <si>
+    <t>Sakamoto (2021) https://doi.org/10.1111/pala.12567 and https://www.sciencedirect.com/science/article/pii/S0960982225008115</t>
+  </si>
+  <si>
+    <t>Rayfield et al. (2001) https://pubmed.ncbi.nlm.nih.gov/11234010/ and https://www.researchgate.net/publication/373284882_Endocranial_anatomy_of_Allosaurus_supports_neural_trends_among_non-avian_theropod_dinosaurs</t>
+  </si>
+  <si>
+    <t>Sakamoto​ (2022) https://peerj.com/articles/13731/ and https://www.researchgate.net/publication/24023506_Estimating_Mass_Properties_of_Dinosaurs_Using_Laser_Imaging_and_3D_Computer_Modelling</t>
+  </si>
+  <si>
+    <t>Sakamoto​ (2022) https://peerj.com/articles/13731/ and https://doi.org/10.1016%2Fj.crpv.2019.09.005</t>
+  </si>
+  <si>
+    <t>Mazzetta et al. (2009) https://www.researchgate.net/publication/240535638_Cranial_Mechanics_and_Functional_Interpretation_of_the_Horned_Carnivorous_Dinosaur_Carnotaurus_sastrei and https://doi.org/10.1016%2Fj.crpv.2019.09.005</t>
+  </si>
+  <si>
+    <t>Sakamoto​ (2022) https://peerj.com/articles/13731/ and https://theropoddatabase.github.io/Ceratosauria.htm#Ceratosaurusnasicornis</t>
+  </si>
+  <si>
+    <t>Sakamoto​ (2022) https://peerj.com/articles/13731/ and https://theropoddatabase.github.io/Dromaeosaurs.htm#Deinonychusantirrhopus</t>
+  </si>
+  <si>
+    <t>Sakamoto​ (2022) https://peerj.com/articles/13731/ and https://pmc.ncbi.nlm.nih.gov/articles/PMC9711522/</t>
+  </si>
+  <si>
+    <t>Sakamoto​ (2022) https://peerj.com/articles/13731/ and https://theropoddatabase.github.io/Carnosauria.htm#Yangchuanosaurusshangyouensis</t>
+  </si>
+  <si>
+    <t>Sakamoto​ (2022) https://peerj.com/articles/13731/ and https://dinoanimals.pl/blogi/czastytanow/walka-o-tron/</t>
+  </si>
+  <si>
+    <t>Sakamoto​ (2022) https://peerj.com/articles/13731/ and https://theropoddatabase.github.io/Dromaeosaurs.htm#Velociraptormongoliensis</t>
+  </si>
+  <si>
+    <t>Sakamoto​ (2022) https://peerj.com/articles/13731/ and https://www.sciencedirect.com/science/article/pii/S0960982225008115</t>
+  </si>
+  <si>
+    <t>Sakamoto​ (2022) https://peerj.com/articles/13731/ and https://theropoddatabase.github.io/Ornithomimosauria.htm#Gallimimusbullatus</t>
+  </si>
+  <si>
+    <t>Sakamoto (2021) https://doi.org/10.1111/pala.12567 and https://gspauldino.com/Trex2022.pdf and https://journals.plos.org/plosbiology/article?id=10.1371/journal.pbio.1001853#s5</t>
+  </si>
+  <si>
+    <t>Sakamoto​ (2022) https://peerj.com/articles/13731/ and https://pmc.ncbi.nlm.nih.gov/articles/PMC10184548</t>
+  </si>
+  <si>
+    <t>Sakamoto (2021) https://doi.org/10.1111/pala.12567 and 5356 and https://doi.org/10.1671/0272-4634(2007)27[108:MTIBTY]2.0.CO;2</t>
+  </si>
 </sst>
 </file>
 
@@ -2897,7 +3032,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2988,6 +3123,12 @@
       <charset val="204"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -3057,7 +3198,7 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -3102,6 +3243,8 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="3" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -6884,6 +7027,267 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000013-5B76-4076-803F-B681175DBE42}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="11"/>
+          <c:order val="11"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Bite force'!$A$381:$H$381</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Theropods</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent6">
+                    <a:lumMod val="60000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent6">
+                    <a:lumMod val="60000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:pPr>
+                      <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                        <a:solidFill>
+                          <a:schemeClr val="tx1">
+                            <a:lumMod val="65000"/>
+                            <a:lumOff val="35000"/>
+                          </a:schemeClr>
+                        </a:solidFill>
+                        <a:latin typeface="+mn-lt"/>
+                        <a:ea typeface="+mn-ea"/>
+                        <a:cs typeface="+mn-cs"/>
+                      </a:defRPr>
+                    </a:pPr>
+                    <a:r>
+                      <a:rPr lang="en-US" baseline="0"/>
+                      <a:t>Theropods:</a:t>
+                    </a:r>
+                  </a:p>
+                  <a:p>
+                    <a:pPr>
+                      <a:defRPr/>
+                    </a:pPr>
+                    <a:r>
+                      <a:rPr lang="en-US" baseline="0"/>
+                      <a:t>y = 0.6966x + 4.158</a:t>
+                    </a:r>
+                    <a:br>
+                      <a:rPr lang="en-US" baseline="0"/>
+                    </a:br>
+                    <a:r>
+                      <a:rPr lang="en-US" baseline="0"/>
+                      <a:t>R² = 0.9226</a:t>
+                    </a:r>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="ru-RU"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Bite force'!$G$382:$G$399</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="18"/>
+                <c:pt idx="0">
+                  <c:v>8.8827664278612932</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>7.3777589082278725</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>7.4633630455200208</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.7905514226139538</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8.9779037737503806</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>8.8827664278612932</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7.3158835045097854</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7.0299729117063858</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8.5221860326488663</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>7.0582932179248807</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>7.3158835045097854</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>5.857933154483459</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2.4965057856313524</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2.5690043578883373</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>7.90100705199242</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>7.7406644019172415</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>6.9206715042486833</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1.8427738320229761</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Bite force'!$H$382:$H$399</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="18"/>
+                <c:pt idx="0">
+                  <c:v>10.953574641928508</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>9.0738331273215191</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8.5705443669132322</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6.7859511064054594</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>10.722816040338978</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>10.789425125735191</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>9.1472569126824954</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8.9676267605024602</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>10.096281793007185</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9.2914731557623504</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>8.1810377046245009</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>7.5688027762846541</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>5.6653745379106697</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>5.9736422887112175</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>9.6931532729655867</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>9.7196426446318274</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>9.5336411039298348</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>5.5200902405130963</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000A-BFF6-48CE-8D2D-9B156A5DC216}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -21134,7 +21538,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{901050C3-4706-4560-809B-127BDF96F50D}">
-  <dimension ref="A1:I380"/>
+  <dimension ref="A1:I413"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="57.28515625" style="10" bestFit="1" customWidth="1"/>
@@ -21157,17 +21561,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="27" t="s">
         <v>220</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
@@ -21199,16 +21603,16 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="27" t="s">
         <v>233</v>
       </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="25"/>
-      <c r="G3" s="26"/>
-      <c r="H3" s="26"/>
+      <c r="B3" s="27"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="27"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28"/>
       <c r="I3" s="13"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -21575,16 +21979,16 @@
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="25" t="s">
+      <c r="A15" s="27" t="s">
         <v>236</v>
       </c>
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="26"/>
-      <c r="H15" s="26"/>
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="28"/>
       <c r="I15" s="13"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -22358,16 +22762,16 @@
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A39" s="25" t="s">
+      <c r="A39" s="27" t="s">
         <v>604</v>
       </c>
-      <c r="B39" s="25"/>
-      <c r="C39" s="25"/>
-      <c r="D39" s="25"/>
-      <c r="E39" s="25"/>
-      <c r="F39" s="25"/>
-      <c r="G39" s="26"/>
-      <c r="H39" s="26"/>
+      <c r="B39" s="27"/>
+      <c r="C39" s="27"/>
+      <c r="D39" s="27"/>
+      <c r="E39" s="27"/>
+      <c r="F39" s="27"/>
+      <c r="G39" s="28"/>
+      <c r="H39" s="28"/>
       <c r="I39" s="16"/>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -23611,16 +24015,16 @@
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A77" s="25" t="s">
+      <c r="A77" s="27" t="s">
         <v>240</v>
       </c>
-      <c r="B77" s="25"/>
-      <c r="C77" s="25"/>
-      <c r="D77" s="25"/>
-      <c r="E77" s="25"/>
-      <c r="F77" s="25"/>
-      <c r="G77" s="26"/>
-      <c r="H77" s="26"/>
+      <c r="B77" s="27"/>
+      <c r="C77" s="27"/>
+      <c r="D77" s="27"/>
+      <c r="E77" s="27"/>
+      <c r="F77" s="27"/>
+      <c r="G77" s="28"/>
+      <c r="H77" s="28"/>
       <c r="I77" s="13"/>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
@@ -24355,16 +24759,16 @@
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A100" s="25" t="s">
+      <c r="A100" s="27" t="s">
         <v>255</v>
       </c>
-      <c r="B100" s="25"/>
-      <c r="C100" s="25"/>
-      <c r="D100" s="25"/>
-      <c r="E100" s="25"/>
-      <c r="F100" s="25"/>
-      <c r="G100" s="26"/>
-      <c r="H100" s="26"/>
+      <c r="B100" s="27"/>
+      <c r="C100" s="27"/>
+      <c r="D100" s="27"/>
+      <c r="E100" s="27"/>
+      <c r="F100" s="27"/>
+      <c r="G100" s="28"/>
+      <c r="H100" s="28"/>
       <c r="I100" s="13"/>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
@@ -26975,16 +27379,16 @@
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A180" s="25" t="s">
+      <c r="A180" s="27" t="s">
         <v>263</v>
       </c>
-      <c r="B180" s="25"/>
-      <c r="C180" s="25"/>
-      <c r="D180" s="25"/>
-      <c r="E180" s="25"/>
-      <c r="F180" s="25"/>
-      <c r="G180" s="26"/>
-      <c r="H180" s="26"/>
+      <c r="B180" s="27"/>
+      <c r="C180" s="27"/>
+      <c r="D180" s="27"/>
+      <c r="E180" s="27"/>
+      <c r="F180" s="27"/>
+      <c r="G180" s="28"/>
+      <c r="H180" s="28"/>
       <c r="I180" s="13"/>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
@@ -29743,16 +30147,16 @@
       </c>
     </row>
     <row r="262" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A262" s="25" t="s">
+      <c r="A262" s="27" t="s">
         <v>318</v>
       </c>
-      <c r="B262" s="25"/>
-      <c r="C262" s="25"/>
-      <c r="D262" s="25"/>
-      <c r="E262" s="25"/>
-      <c r="F262" s="25"/>
-      <c r="G262" s="26"/>
-      <c r="H262" s="26"/>
+      <c r="B262" s="27"/>
+      <c r="C262" s="27"/>
+      <c r="D262" s="27"/>
+      <c r="E262" s="27"/>
+      <c r="F262" s="27"/>
+      <c r="G262" s="28"/>
+      <c r="H262" s="28"/>
     </row>
     <row r="263" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A263" s="2" t="s">
@@ -29854,16 +30258,16 @@
       </c>
     </row>
     <row r="266" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A266" s="25" t="s">
+      <c r="A266" s="27" t="s">
         <v>218</v>
       </c>
-      <c r="B266" s="25"/>
-      <c r="C266" s="25"/>
-      <c r="D266" s="25"/>
-      <c r="E266" s="25"/>
-      <c r="F266" s="25"/>
-      <c r="G266" s="26"/>
-      <c r="H266" s="26"/>
+      <c r="B266" s="27"/>
+      <c r="C266" s="27"/>
+      <c r="D266" s="27"/>
+      <c r="E266" s="27"/>
+      <c r="F266" s="27"/>
+      <c r="G266" s="28"/>
+      <c r="H266" s="28"/>
     </row>
     <row r="267" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A267" s="2" t="s">
@@ -31351,16 +31755,16 @@
       </c>
     </row>
     <row r="312" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A312" s="25" t="s">
+      <c r="A312" s="27" t="s">
         <v>361</v>
       </c>
-      <c r="B312" s="25"/>
-      <c r="C312" s="25"/>
-      <c r="D312" s="25"/>
-      <c r="E312" s="25"/>
-      <c r="F312" s="25"/>
-      <c r="G312" s="26"/>
-      <c r="H312" s="26"/>
+      <c r="B312" s="27"/>
+      <c r="C312" s="27"/>
+      <c r="D312" s="27"/>
+      <c r="E312" s="27"/>
+      <c r="F312" s="27"/>
+      <c r="G312" s="28"/>
+      <c r="H312" s="28"/>
       <c r="I312" s="3"/>
     </row>
     <row r="313" spans="1:9" x14ac:dyDescent="0.25">
@@ -32168,19 +32572,19 @@
         <v>1.5835439013324151</v>
       </c>
     </row>
-    <row r="337" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A337" s="25" t="s">
+    <row r="337" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A337" s="27" t="s">
         <v>388</v>
       </c>
-      <c r="B337" s="25"/>
-      <c r="C337" s="25"/>
-      <c r="D337" s="25"/>
-      <c r="E337" s="25"/>
-      <c r="F337" s="25"/>
-      <c r="G337" s="26"/>
-      <c r="H337" s="26"/>
-    </row>
-    <row r="338" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B337" s="27"/>
+      <c r="C337" s="27"/>
+      <c r="D337" s="27"/>
+      <c r="E337" s="27"/>
+      <c r="F337" s="27"/>
+      <c r="G337" s="28"/>
+      <c r="H337" s="28"/>
+    </row>
+    <row r="338" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A338" s="2" t="s">
         <v>21</v>
       </c>
@@ -32208,8 +32612,11 @@
         <f t="shared" si="40"/>
         <v>7.4719320782451222</v>
       </c>
-    </row>
-    <row r="339" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I338" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="339" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A339" s="2" t="s">
         <v>23</v>
       </c>
@@ -32237,8 +32644,11 @@
         <f t="shared" si="40"/>
         <v>8.6762648860214249</v>
       </c>
-    </row>
-    <row r="340" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I339" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="340" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A340" s="2" t="s">
         <v>0</v>
       </c>
@@ -32266,20 +32676,23 @@
         <f t="shared" si="40"/>
         <v>3.912023005428146</v>
       </c>
-    </row>
-    <row r="341" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A341" s="25" t="s">
+      <c r="I340" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="341" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A341" s="27" t="s">
         <v>397</v>
       </c>
-      <c r="B341" s="25"/>
-      <c r="C341" s="25"/>
-      <c r="D341" s="25"/>
-      <c r="E341" s="25"/>
-      <c r="F341" s="25"/>
-      <c r="G341" s="26"/>
-      <c r="H341" s="26"/>
-    </row>
-    <row r="342" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B341" s="27"/>
+      <c r="C341" s="27"/>
+      <c r="D341" s="27"/>
+      <c r="E341" s="27"/>
+      <c r="F341" s="27"/>
+      <c r="G341" s="28"/>
+      <c r="H341" s="28"/>
+    </row>
+    <row r="342" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A342" s="2" t="s">
         <v>398</v>
       </c>
@@ -32308,8 +32721,12 @@
         <f t="shared" si="42"/>
         <v>3.3816730156477139</v>
       </c>
-    </row>
-    <row r="343" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I342" s="3">
+        <f>C342/EXP(0.7444*LN(B342)+6.5696)</f>
+        <v>0.52278019346902327</v>
+      </c>
+    </row>
+    <row r="343" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A343" s="2" t="s">
         <v>398</v>
       </c>
@@ -32338,8 +32755,12 @@
         <f t="shared" si="42"/>
         <v>4.6626068611097784</v>
       </c>
-    </row>
-    <row r="344" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I343" s="3">
+        <f t="shared" ref="I343:I380" si="43">C343/EXP(0.7444*LN(B343)+6.5696)</f>
+        <v>0.76805211235176341</v>
+      </c>
+    </row>
+    <row r="344" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A344" s="2" t="s">
         <v>398</v>
       </c>
@@ -32368,8 +32789,12 @@
         <f t="shared" si="42"/>
         <v>5.4527463076570335</v>
       </c>
-    </row>
-    <row r="345" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I344" s="3">
+        <f t="shared" si="43"/>
+        <v>1.3436132286805722</v>
+      </c>
+    </row>
+    <row r="345" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A345" s="2" t="s">
         <v>398</v>
       </c>
@@ -32398,8 +32823,12 @@
         <f t="shared" si="42"/>
         <v>5.1734324848757689</v>
       </c>
-    </row>
-    <row r="346" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I345" s="3">
+        <f t="shared" si="43"/>
+        <v>1.0161780721113571</v>
+      </c>
+    </row>
+    <row r="346" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A346" s="2" t="s">
         <v>398</v>
       </c>
@@ -32428,8 +32857,12 @@
         <f t="shared" si="42"/>
         <v>5.3649706967746473</v>
       </c>
-    </row>
-    <row r="347" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I346" s="3">
+        <f t="shared" si="43"/>
+        <v>1.1729762689457426</v>
+      </c>
+    </row>
+    <row r="347" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A347" s="2" t="s">
         <v>398</v>
       </c>
@@ -32458,8 +32891,12 @@
         <f t="shared" si="42"/>
         <v>5.2585902932160762</v>
       </c>
-    </row>
-    <row r="348" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I347" s="3">
+        <f t="shared" si="43"/>
+        <v>0.96607504938535083</v>
+      </c>
+    </row>
+    <row r="348" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A348" s="2" t="s">
         <v>398</v>
       </c>
@@ -32488,8 +32925,12 @@
         <f t="shared" si="42"/>
         <v>5.723478821795041</v>
       </c>
-    </row>
-    <row r="349" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I348" s="3">
+        <f t="shared" si="43"/>
+        <v>1.4544360599992894</v>
+      </c>
+    </row>
+    <row r="349" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A349" s="2" t="s">
         <v>398</v>
       </c>
@@ -32518,8 +32959,12 @@
         <f t="shared" si="42"/>
         <v>5.6942084394949273</v>
       </c>
-    </row>
-    <row r="350" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I349" s="3">
+        <f t="shared" si="43"/>
+        <v>1.1694879014336035</v>
+      </c>
+    </row>
+    <row r="350" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A350" s="2" t="s">
         <v>398</v>
       </c>
@@ -32548,8 +32993,12 @@
         <f t="shared" si="42"/>
         <v>5.4979285304502659</v>
       </c>
-    </row>
-    <row r="351" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I350" s="3">
+        <f t="shared" si="43"/>
+        <v>0.86053774613407863</v>
+      </c>
+    </row>
+    <row r="351" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A351" s="2" t="s">
         <v>398</v>
       </c>
@@ -32578,8 +33027,12 @@
         <f t="shared" si="42"/>
         <v>5.5099047214969818</v>
       </c>
-    </row>
-    <row r="352" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I351" s="3">
+        <f t="shared" si="43"/>
+        <v>0.80936895884482152</v>
+      </c>
+    </row>
+    <row r="352" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A352" s="2" t="s">
         <v>398</v>
       </c>
@@ -32608,8 +33061,12 @@
         <f t="shared" si="42"/>
         <v>5.9414809736088321</v>
       </c>
-    </row>
-    <row r="353" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I352" s="3">
+        <f t="shared" si="43"/>
+        <v>1.1657545538706269</v>
+      </c>
+    </row>
+    <row r="353" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A353" s="2" t="s">
         <v>398</v>
       </c>
@@ -32638,8 +33095,12 @@
         <f t="shared" si="42"/>
         <v>5.8211172913589566</v>
       </c>
-    </row>
-    <row r="354" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I353" s="3">
+        <f t="shared" si="43"/>
+        <v>0.97218111508073835</v>
+      </c>
+    </row>
+    <row r="354" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A354" s="2" t="s">
         <v>398</v>
       </c>
@@ -32668,8 +33129,12 @@
         <f t="shared" si="42"/>
         <v>5.87211984581133</v>
       </c>
-    </row>
-    <row r="355" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I354" s="3">
+        <f t="shared" si="43"/>
+        <v>0.98472453838656349</v>
+      </c>
+    </row>
+    <row r="355" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A355" s="2" t="s">
         <v>398</v>
       </c>
@@ -32698,8 +33163,12 @@
         <f t="shared" si="42"/>
         <v>6.0626945443620048</v>
       </c>
-    </row>
-    <row r="356" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I355" s="3">
+        <f t="shared" si="43"/>
+        <v>1.0914462737832678</v>
+      </c>
+    </row>
+    <row r="356" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A356" s="2" t="s">
         <v>398</v>
       </c>
@@ -32728,8 +33197,12 @@
         <f t="shared" si="42"/>
         <v>5.8269144090432832</v>
       </c>
-    </row>
-    <row r="357" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I356" s="3">
+        <f t="shared" si="43"/>
+        <v>0.68413720744584661</v>
+      </c>
+    </row>
+    <row r="357" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A357" s="2" t="s">
         <v>398</v>
       </c>
@@ -32758,8 +33231,12 @@
         <f t="shared" si="42"/>
         <v>6.3656700329832843</v>
       </c>
-    </row>
-    <row r="358" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I357" s="3">
+        <f t="shared" si="43"/>
+        <v>1.1342408010756679</v>
+      </c>
+    </row>
+    <row r="358" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A358" s="2" t="s">
         <v>398</v>
       </c>
@@ -32781,15 +33258,19 @@
         <v>399</v>
       </c>
       <c r="G358" s="3">
-        <f t="shared" ref="G358:H380" si="43">LN(B358)</f>
+        <f t="shared" ref="G358:H380" si="44">LN(B358)</f>
         <v>-0.40047756659712525</v>
       </c>
       <c r="H358" s="3">
+        <f t="shared" si="44"/>
+        <v>6.1332083286896628</v>
+      </c>
+      <c r="I358" s="3">
         <f t="shared" si="43"/>
-        <v>6.1332083286896628</v>
-      </c>
-    </row>
-    <row r="359" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.87085815299587077</v>
+      </c>
+    </row>
+    <row r="359" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A359" s="2" t="s">
         <v>398</v>
       </c>
@@ -32811,15 +33292,19 @@
         <v>399</v>
       </c>
       <c r="G359" s="3">
+        <f t="shared" si="44"/>
+        <v>-0.35667494393873245</v>
+      </c>
+      <c r="H359" s="3">
+        <f t="shared" si="44"/>
+        <v>6.170791039838706</v>
+      </c>
+      <c r="I359" s="3">
         <f t="shared" si="43"/>
-        <v>-0.35667494393873245</v>
-      </c>
-      <c r="H359" s="3">
-        <f t="shared" si="43"/>
-        <v>6.170791039838706</v>
-      </c>
-    </row>
-    <row r="360" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.87520237653978916</v>
+      </c>
+    </row>
+    <row r="360" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A360" s="2" t="s">
         <v>398</v>
       </c>
@@ -32841,15 +33326,19 @@
         <v>399</v>
       </c>
       <c r="G360" s="3">
+        <f t="shared" si="44"/>
+        <v>-0.2744368457017603</v>
+      </c>
+      <c r="H360" s="3">
+        <f t="shared" si="44"/>
+        <v>6.4681596524701694</v>
+      </c>
+      <c r="I360" s="3">
         <f t="shared" si="43"/>
-        <v>-0.2744368457017603</v>
-      </c>
-      <c r="H360" s="3">
-        <f t="shared" si="43"/>
-        <v>6.4681596524701694</v>
-      </c>
-    </row>
-    <row r="361" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1.1083256359527567</v>
+      </c>
+    </row>
+    <row r="361" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A361" s="2" t="s">
         <v>398</v>
       </c>
@@ -32871,15 +33360,19 @@
         <v>399</v>
       </c>
       <c r="G361" s="3">
+        <f t="shared" si="44"/>
+        <v>-2.0202707317519466E-2</v>
+      </c>
+      <c r="H361" s="3">
+        <f t="shared" si="44"/>
+        <v>6.4862596941137873</v>
+      </c>
+      <c r="I361" s="3">
         <f t="shared" si="43"/>
-        <v>-2.0202707317519466E-2</v>
-      </c>
-      <c r="H361" s="3">
-        <f t="shared" si="43"/>
-        <v>6.4862596941137873</v>
-      </c>
-    </row>
-    <row r="362" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.93397892003930871</v>
+      </c>
+    </row>
+    <row r="362" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A362" s="2" t="s">
         <v>398</v>
       </c>
@@ -32901,15 +33394,19 @@
         <v>399</v>
       </c>
       <c r="G362" s="3">
+        <f t="shared" si="44"/>
+        <v>0</v>
+      </c>
+      <c r="H362" s="3">
+        <f t="shared" si="44"/>
+        <v>6.7327460101273005</v>
+      </c>
+      <c r="I362" s="3">
         <f t="shared" si="43"/>
-        <v>0</v>
-      </c>
-      <c r="H362" s="3">
-        <f t="shared" si="43"/>
-        <v>6.7327460101273005</v>
-      </c>
-    </row>
-    <row r="363" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1.1772085615125738</v>
+      </c>
+    </row>
+    <row r="363" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A363" s="2" t="s">
         <v>398</v>
       </c>
@@ -32931,15 +33428,19 @@
         <v>399</v>
       </c>
       <c r="G363" s="3">
+        <f t="shared" si="44"/>
+        <v>0.131028262406404</v>
+      </c>
+      <c r="H363" s="3">
+        <f t="shared" si="44"/>
+        <v>6.2476761825269209</v>
+      </c>
+      <c r="I363" s="3">
         <f t="shared" si="43"/>
-        <v>0.131028262406404</v>
-      </c>
-      <c r="H363" s="3">
-        <f t="shared" si="43"/>
-        <v>6.2476761825269209</v>
-      </c>
-    </row>
-    <row r="364" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.65740089521085987</v>
+      </c>
+    </row>
+    <row r="364" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A364" s="2" t="s">
         <v>398</v>
       </c>
@@ -32961,15 +33462,19 @@
         <v>399</v>
       </c>
       <c r="G364" s="3">
+        <f t="shared" si="44"/>
+        <v>0.36464311358790924</v>
+      </c>
+      <c r="H364" s="3">
+        <f t="shared" si="44"/>
+        <v>6.8369376185801451</v>
+      </c>
+      <c r="I364" s="3">
         <f t="shared" si="43"/>
-        <v>0.36464311358790924</v>
-      </c>
-      <c r="H364" s="3">
-        <f t="shared" si="43"/>
-        <v>6.8369376185801451</v>
-      </c>
-    </row>
-    <row r="365" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.99590568946333324</v>
+      </c>
+    </row>
+    <row r="365" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A365" s="2" t="s">
         <v>398</v>
       </c>
@@ -32991,15 +33496,19 @@
         <v>399</v>
       </c>
       <c r="G365" s="3">
+        <f t="shared" si="44"/>
+        <v>0.45742484703887548</v>
+      </c>
+      <c r="H365" s="3">
+        <f t="shared" si="44"/>
+        <v>7.2528740265556051</v>
+      </c>
+      <c r="I365" s="3">
         <f t="shared" si="43"/>
-        <v>0.45742484703887548</v>
-      </c>
-      <c r="H365" s="3">
-        <f t="shared" si="43"/>
-        <v>7.2528740265556051</v>
-      </c>
-    </row>
-    <row r="366" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1.4088404221794428</v>
+      </c>
+    </row>
+    <row r="366" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A366" s="2" t="s">
         <v>398</v>
       </c>
@@ -33021,15 +33530,19 @@
         <v>399</v>
       </c>
       <c r="G366" s="3">
+        <f t="shared" si="44"/>
+        <v>0.5709795465857378</v>
+      </c>
+      <c r="H366" s="3">
+        <f t="shared" si="44"/>
+        <v>7.184624926021498</v>
+      </c>
+      <c r="I366" s="3">
         <f t="shared" si="43"/>
-        <v>0.5709795465857378</v>
-      </c>
-      <c r="H366" s="3">
-        <f t="shared" si="43"/>
-        <v>7.184624926021498</v>
-      </c>
-    </row>
-    <row r="367" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1.2092347863063504</v>
+      </c>
+    </row>
+    <row r="367" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A367" s="2" t="s">
         <v>398</v>
       </c>
@@ -33051,15 +33564,19 @@
         <v>399</v>
       </c>
       <c r="G367" s="3">
+        <f t="shared" si="44"/>
+        <v>0.65232518603969014</v>
+      </c>
+      <c r="H367" s="3">
+        <f t="shared" si="44"/>
+        <v>7.0730493499602378</v>
+      </c>
+      <c r="I367" s="3">
         <f t="shared" si="43"/>
-        <v>0.65232518603969014</v>
-      </c>
-      <c r="H367" s="3">
-        <f t="shared" si="43"/>
-        <v>7.0730493499602378</v>
-      </c>
-    </row>
-    <row r="368" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1.018018897659553</v>
+      </c>
+    </row>
+    <row r="368" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A368" s="2" t="s">
         <v>398</v>
       </c>
@@ -33081,15 +33598,19 @@
         <v>399</v>
       </c>
       <c r="G368" s="3">
+        <f t="shared" si="44"/>
+        <v>0.72754860727727766</v>
+      </c>
+      <c r="H368" s="3">
+        <f t="shared" si="44"/>
+        <v>7.4760175778698148</v>
+      </c>
+      <c r="I368" s="3">
         <f t="shared" si="43"/>
-        <v>0.72754860727727766</v>
-      </c>
-      <c r="H368" s="3">
-        <f t="shared" si="43"/>
-        <v>7.4760175778698148</v>
-      </c>
-    </row>
-    <row r="369" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1.4402697099305548</v>
+      </c>
+    </row>
+    <row r="369" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A369" s="2" t="s">
         <v>398</v>
       </c>
@@ -33111,15 +33632,19 @@
         <v>399</v>
       </c>
       <c r="G369" s="3">
+        <f t="shared" si="44"/>
+        <v>0.73716406597671957</v>
+      </c>
+      <c r="H369" s="3">
+        <f t="shared" si="44"/>
+        <v>7.3644650919640675</v>
+      </c>
+      <c r="I369" s="3">
         <f t="shared" si="43"/>
-        <v>0.73716406597671957</v>
-      </c>
-      <c r="H369" s="3">
-        <f t="shared" si="43"/>
-        <v>7.3644650919640675</v>
-      </c>
-    </row>
-    <row r="370" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1.2790532569476043</v>
+      </c>
+    </row>
+    <row r="370" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A370" s="2" t="s">
         <v>398</v>
       </c>
@@ -33141,15 +33666,19 @@
         <v>399</v>
       </c>
       <c r="G370" s="3">
+        <f t="shared" si="44"/>
+        <v>0.75141608868392118</v>
+      </c>
+      <c r="H370" s="3">
+        <f t="shared" si="44"/>
+        <v>7.184624926021498</v>
+      </c>
+      <c r="I370" s="3">
         <f t="shared" si="43"/>
-        <v>0.75141608868392118</v>
-      </c>
-      <c r="H370" s="3">
-        <f t="shared" si="43"/>
-        <v>7.184624926021498</v>
-      </c>
-    </row>
-    <row r="371" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1.0572495688902517</v>
+      </c>
+    </row>
+    <row r="371" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A371" s="2" t="s">
         <v>400</v>
       </c>
@@ -33171,15 +33700,19 @@
         <v>401</v>
       </c>
       <c r="G371" s="3">
+        <f t="shared" si="44"/>
+        <v>-2.1856913415225465</v>
+      </c>
+      <c r="H371" s="3">
+        <f t="shared" si="44"/>
+        <v>5.0369526024136295</v>
+      </c>
+      <c r="I371" s="3">
         <f t="shared" si="43"/>
-        <v>-2.1856913415225465</v>
-      </c>
-      <c r="H371" s="3">
-        <f t="shared" si="43"/>
-        <v>5.0369526024136295</v>
-      </c>
-    </row>
-    <row r="372" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1.0989786374296873</v>
+      </c>
+    </row>
+    <row r="372" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A372" s="2" t="s">
         <v>402</v>
       </c>
@@ -33201,15 +33734,19 @@
         <v>401</v>
       </c>
       <c r="G372" s="3">
+        <f t="shared" si="44"/>
+        <v>-3.4900285953687713</v>
+      </c>
+      <c r="H372" s="3">
+        <f t="shared" si="44"/>
+        <v>4.4402955427978572</v>
+      </c>
+      <c r="I372" s="3">
         <f t="shared" si="43"/>
-        <v>-3.4900285953687713</v>
-      </c>
-      <c r="H372" s="3">
-        <f t="shared" si="43"/>
-        <v>4.4402955427978572</v>
-      </c>
-    </row>
-    <row r="373" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1.5978721361061514</v>
+      </c>
+    </row>
+    <row r="373" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A373" s="2" t="s">
         <v>403</v>
       </c>
@@ -33231,15 +33768,19 @@
         <v>401</v>
       </c>
       <c r="G373" s="3">
+        <f t="shared" si="44"/>
+        <v>-1.8585405029184061</v>
+      </c>
+      <c r="H373" s="3">
+        <f t="shared" si="44"/>
+        <v>4.8559289043352747</v>
+      </c>
+      <c r="I373" s="3">
         <f t="shared" si="43"/>
-        <v>-1.8585405029184061</v>
-      </c>
-      <c r="H373" s="3">
-        <f t="shared" si="43"/>
-        <v>4.8559289043352747</v>
-      </c>
-    </row>
-    <row r="374" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.7187989784281269</v>
+      </c>
+    </row>
+    <row r="374" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A374" s="2" t="s">
         <v>404</v>
       </c>
@@ -33261,15 +33802,19 @@
         <v>401</v>
       </c>
       <c r="G374" s="3">
+        <f t="shared" si="44"/>
+        <v>-1.1727971868574862</v>
+      </c>
+      <c r="H374" s="3">
+        <f t="shared" si="44"/>
+        <v>5.2062020776402314</v>
+      </c>
+      <c r="I374" s="3">
         <f t="shared" si="43"/>
-        <v>-1.1727971868574862</v>
-      </c>
-      <c r="H374" s="3">
-        <f t="shared" si="43"/>
-        <v>5.2062020776402314</v>
-      </c>
-    </row>
-    <row r="375" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.61240117503477931</v>
+      </c>
+    </row>
+    <row r="375" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A375" s="2" t="s">
         <v>405</v>
       </c>
@@ -33291,15 +33836,19 @@
         <v>401</v>
       </c>
       <c r="G375" s="3">
+        <f t="shared" si="44"/>
+        <v>-4.2758664388454912</v>
+      </c>
+      <c r="H375" s="3">
+        <f t="shared" si="44"/>
+        <v>3.9684033388642534</v>
+      </c>
+      <c r="I375" s="3">
         <f t="shared" si="43"/>
-        <v>-4.2758664388454912</v>
-      </c>
-      <c r="H375" s="3">
-        <f t="shared" si="43"/>
-        <v>3.9684033388642534</v>
-      </c>
-    </row>
-    <row r="376" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1.7891816131378486</v>
+      </c>
+    </row>
+    <row r="376" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A376" s="2" t="s">
         <v>406</v>
       </c>
@@ -33321,15 +33870,19 @@
         <v>401</v>
       </c>
       <c r="G376" s="3">
+        <f t="shared" si="44"/>
+        <v>-1.9980459034758418</v>
+      </c>
+      <c r="H376" s="3">
+        <f t="shared" si="44"/>
+        <v>4.8835592115282793</v>
+      </c>
+      <c r="I376" s="3">
         <f t="shared" si="43"/>
-        <v>-1.9980459034758418</v>
-      </c>
-      <c r="H376" s="3">
-        <f t="shared" si="43"/>
-        <v>4.8835592115282793</v>
-      </c>
-    </row>
-    <row r="377" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.81979955155935336</v>
+      </c>
+    </row>
+    <row r="377" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A377" s="2" t="s">
         <v>407</v>
       </c>
@@ -33351,15 +33904,19 @@
         <v>408</v>
       </c>
       <c r="G377" s="3">
+        <f t="shared" si="44"/>
+        <v>-6.7944265936751336</v>
+      </c>
+      <c r="H377" s="3">
+        <f t="shared" si="44"/>
+        <v>0.26236426446749106</v>
+      </c>
+      <c r="I377" s="3">
         <f t="shared" si="43"/>
-        <v>-6.7944265936751336</v>
-      </c>
-      <c r="H377" s="3">
-        <f t="shared" si="43"/>
-        <v>0.26236426446749106</v>
-      </c>
-    </row>
-    <row r="378" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.28665823856179024</v>
+      </c>
+    </row>
+    <row r="378" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A378" s="2" t="s">
         <v>409</v>
       </c>
@@ -33381,15 +33938,19 @@
         <v>410</v>
       </c>
       <c r="G378" s="3">
+        <f t="shared" si="44"/>
+        <v>-6.6002705792341763</v>
+      </c>
+      <c r="H378" s="3">
+        <f t="shared" si="44"/>
+        <v>1.8718021769015913</v>
+      </c>
+      <c r="I378" s="3">
         <f t="shared" si="43"/>
-        <v>-6.6002705792341763</v>
-      </c>
-      <c r="H378" s="3">
-        <f t="shared" si="43"/>
-        <v>1.8718021769015913</v>
-      </c>
-    </row>
-    <row r="379" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1.2404120168541442</v>
+      </c>
+    </row>
+    <row r="379" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A379" s="2" t="s">
         <v>409</v>
       </c>
@@ -33411,15 +33972,19 @@
         <v>410</v>
       </c>
       <c r="G379" s="3">
+        <f t="shared" si="44"/>
+        <v>-7.5055922797377574</v>
+      </c>
+      <c r="H379" s="3">
+        <f t="shared" si="44"/>
+        <v>0.47000362924573563</v>
+      </c>
+      <c r="I379" s="3">
         <f t="shared" si="43"/>
-        <v>-7.5055922797377574</v>
-      </c>
-      <c r="H379" s="3">
-        <f t="shared" si="43"/>
-        <v>0.47000362924573563</v>
-      </c>
-    </row>
-    <row r="380" spans="1:8" x14ac:dyDescent="0.25">
+        <v>0.59903606277191157</v>
+      </c>
+    </row>
+    <row r="380" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A380" s="2" t="s">
         <v>411</v>
       </c>
@@ -33441,21 +34006,1010 @@
         <v>412</v>
       </c>
       <c r="G380" s="3">
+        <f t="shared" si="44"/>
+        <v>-9.8081773727318033</v>
+      </c>
+      <c r="H380" s="3">
+        <f t="shared" si="44"/>
+        <v>0.33647223662121289</v>
+      </c>
+      <c r="I380" s="3">
         <f t="shared" si="43"/>
-        <v>-9.8081773727318033</v>
-      </c>
-      <c r="H380" s="3">
-        <f t="shared" si="43"/>
-        <v>0.33647223662121289</v>
-      </c>
+        <v>2.9097858077284147</v>
+      </c>
+    </row>
+    <row r="381" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A381" s="27" t="s">
+        <v>649</v>
+      </c>
+      <c r="B381" s="27"/>
+      <c r="C381" s="27"/>
+      <c r="D381" s="27"/>
+      <c r="E381" s="27"/>
+      <c r="F381" s="27"/>
+      <c r="G381" s="28"/>
+      <c r="H381" s="28"/>
+    </row>
+    <row r="382" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A382" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B382" s="3">
+        <v>7206.7</v>
+      </c>
+      <c r="C382" s="3">
+        <v>57158</v>
+      </c>
+      <c r="D382" s="3">
+        <f>C382*(1/B382)^(2/3)</f>
+        <v>153.19787043999401</v>
+      </c>
+      <c r="E382" s="25" t="s">
+        <v>237</v>
+      </c>
+      <c r="F382" s="25" t="s">
+        <v>662</v>
+      </c>
+      <c r="G382" s="3">
+        <f t="shared" ref="G382" si="45">LN(B382)</f>
+        <v>8.8827664278612932</v>
+      </c>
+      <c r="H382" s="3">
+        <f t="shared" ref="H382" si="46">LN(C382)</f>
+        <v>10.953574641928508</v>
+      </c>
+      <c r="I382" s="3">
+        <f t="shared" ref="I382:I409" si="47">C382/EXP(0.6966*LN(B382)+4.158)</f>
+        <v>1.8364595276640094</v>
+      </c>
+    </row>
+    <row r="383" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A383" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B383" s="3">
+        <v>1600</v>
+      </c>
+      <c r="C383" s="3">
+        <v>8724</v>
+      </c>
+      <c r="D383" s="3">
+        <f>C383*(1/B383)^(2/3)</f>
+        <v>63.772826870422612</v>
+      </c>
+      <c r="E383" s="25" t="s">
+        <v>237</v>
+      </c>
+      <c r="F383" s="25" t="s">
+        <v>674</v>
+      </c>
+      <c r="G383" s="3">
+        <f t="shared" ref="G383:G399" si="48">LN(B383)</f>
+        <v>7.3777589082278725</v>
+      </c>
+      <c r="H383" s="3">
+        <f t="shared" ref="H383:H399" si="49">LN(C383)</f>
+        <v>9.0738331273215191</v>
+      </c>
+      <c r="I383" s="3">
+        <f t="shared" si="47"/>
+        <v>0.79970391333694757</v>
+      </c>
+    </row>
+    <row r="384" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A384" s="2" t="s">
+        <v>651</v>
+      </c>
+      <c r="B384" s="3">
+        <v>1743</v>
+      </c>
+      <c r="C384" s="3">
+        <v>5274</v>
+      </c>
+      <c r="D384" s="3">
+        <f>C384*(1/B384)^(2/3)</f>
+        <v>36.414571236413259</v>
+      </c>
+      <c r="E384" s="25" t="s">
+        <v>661</v>
+      </c>
+      <c r="F384" s="25" t="s">
+        <v>682</v>
+      </c>
+      <c r="G384" s="3">
+        <f t="shared" si="48"/>
+        <v>7.4633630455200208</v>
+      </c>
+      <c r="H384" s="3">
+        <f t="shared" si="49"/>
+        <v>8.5705443669132322</v>
+      </c>
+      <c r="I384" s="3">
+        <f t="shared" si="47"/>
+        <v>0.45546594430618215</v>
+      </c>
+    </row>
+    <row r="385" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A385" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="B385" s="3">
+        <v>16.29</v>
+      </c>
+      <c r="C385" s="3">
+        <v>885.32172179999998</v>
+      </c>
+      <c r="D385" s="3">
+        <f>C385*(1/B385)^(2/3)</f>
+        <v>137.76970562343334</v>
+      </c>
+      <c r="E385" s="25" t="s">
+        <v>661</v>
+      </c>
+      <c r="F385" s="25" t="s">
+        <v>693</v>
+      </c>
+      <c r="G385" s="3">
+        <f t="shared" si="48"/>
+        <v>2.7905514226139538</v>
+      </c>
+      <c r="H385" s="3">
+        <f t="shared" si="49"/>
+        <v>6.7859511064054594</v>
+      </c>
+      <c r="I385" s="3">
+        <f>C385/EXP(0.6966*LN(B385)+4.158)</f>
+        <v>1.9818940639496714</v>
+      </c>
+    </row>
+    <row r="386" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A386" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B386" s="3">
+        <v>7926</v>
+      </c>
+      <c r="C386" s="3">
+        <v>45379.513619999998</v>
+      </c>
+      <c r="D386" s="3">
+        <f>C386*(1/B386)^(2/3)</f>
+        <v>114.15382236109754</v>
+      </c>
+      <c r="E386" s="25" t="s">
+        <v>661</v>
+      </c>
+      <c r="F386" s="25" t="s">
+        <v>663</v>
+      </c>
+      <c r="G386" s="3">
+        <f t="shared" si="48"/>
+        <v>8.9779037737503806</v>
+      </c>
+      <c r="H386" s="3">
+        <f t="shared" si="49"/>
+        <v>10.722816040338978</v>
+      </c>
+      <c r="I386" s="3">
+        <f t="shared" si="47"/>
+        <v>1.3645275773397363</v>
+      </c>
+    </row>
+    <row r="387" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A387" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B387" s="3">
+        <v>7206.7</v>
+      </c>
+      <c r="C387" s="3">
+        <v>48505.143640000002</v>
+      </c>
+      <c r="D387" s="3">
+        <f>C387*(1/B387)^(2/3)</f>
+        <v>130.00603084492144</v>
+      </c>
+      <c r="E387" s="25" t="s">
+        <v>661</v>
+      </c>
+      <c r="F387" s="25" t="s">
+        <v>675</v>
+      </c>
+      <c r="G387" s="3">
+        <f t="shared" si="48"/>
+        <v>8.8827664278612932</v>
+      </c>
+      <c r="H387" s="3">
+        <f t="shared" si="49"/>
+        <v>10.789425125735191</v>
+      </c>
+      <c r="I387" s="3">
+        <f t="shared" si="47"/>
+        <v>1.5584473420761631</v>
+      </c>
+    </row>
+    <row r="388" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A388" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B388" s="3">
+        <v>1504</v>
+      </c>
+      <c r="C388" s="3">
+        <v>9388.6511339999997</v>
+      </c>
+      <c r="D388" s="3">
+        <f>C388*(1/B388)^(2/3)</f>
+        <v>71.521724521333155</v>
+      </c>
+      <c r="E388" s="25" t="s">
+        <v>661</v>
+      </c>
+      <c r="F388" s="25" t="s">
+        <v>650</v>
+      </c>
+      <c r="G388" s="3">
+        <f t="shared" si="48"/>
+        <v>7.3158835045097854</v>
+      </c>
+      <c r="H388" s="3">
+        <f t="shared" si="49"/>
+        <v>9.1472569126824954</v>
+      </c>
+      <c r="I388" s="3">
+        <f t="shared" si="47"/>
+        <v>0.89853687178178665</v>
+      </c>
+    </row>
+    <row r="389" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A389" s="2" t="s">
+        <v>653</v>
+      </c>
+      <c r="B389" s="3">
+        <v>1130</v>
+      </c>
+      <c r="C389" s="3">
+        <v>7844.9615229999999</v>
+      </c>
+      <c r="D389" s="3">
+        <f>C389*(1/B389)^(2/3)</f>
+        <v>72.311136759110411</v>
+      </c>
+      <c r="E389" s="25" t="s">
+        <v>661</v>
+      </c>
+      <c r="F389" s="25" t="s">
+        <v>650</v>
+      </c>
+      <c r="G389" s="3">
+        <f t="shared" si="48"/>
+        <v>7.0299729117063858</v>
+      </c>
+      <c r="H389" s="3">
+        <f t="shared" si="49"/>
+        <v>8.9676267605024602</v>
+      </c>
+      <c r="I389" s="3">
+        <f t="shared" si="47"/>
+        <v>0.91626251238541745</v>
+      </c>
+    </row>
+    <row r="390" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A390" s="2" t="s">
+        <v>654</v>
+      </c>
+      <c r="B390" s="3">
+        <f>POWER(10,2.754*LOG(480)-0.683)/1000</f>
+        <v>5025.0266311715559</v>
+      </c>
+      <c r="C390" s="3">
+        <v>24252.665140000001</v>
+      </c>
+      <c r="D390" s="3">
+        <f>C390*(1/B390)^(2/3)</f>
+        <v>82.667326383280667</v>
+      </c>
+      <c r="E390" s="25" t="s">
+        <v>661</v>
+      </c>
+      <c r="F390" s="25" t="s">
+        <v>691</v>
+      </c>
+      <c r="G390" s="3">
+        <f t="shared" si="48"/>
+        <v>8.5221860326488663</v>
+      </c>
+      <c r="H390" s="3">
+        <f t="shared" si="49"/>
+        <v>10.096281793007185</v>
+      </c>
+      <c r="I390" s="3">
+        <f t="shared" si="47"/>
+        <v>1.0017284947919318</v>
+      </c>
+    </row>
+    <row r="391" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A391" s="2" t="s">
+        <v>655</v>
+      </c>
+      <c r="B391" s="3">
+        <v>1162.45940674742</v>
+      </c>
+      <c r="C391" s="3">
+        <v>10845.148929999999</v>
+      </c>
+      <c r="D391" s="3">
+        <f>C391*(1/B391)^(2/3)</f>
+        <v>98.095779558141302</v>
+      </c>
+      <c r="E391" s="25" t="s">
+        <v>661</v>
+      </c>
+      <c r="F391" s="25" t="s">
+        <v>650</v>
+      </c>
+      <c r="G391" s="3">
+        <f t="shared" si="48"/>
+        <v>7.0582932179248807</v>
+      </c>
+      <c r="H391" s="3">
+        <f t="shared" si="49"/>
+        <v>9.2914731557623504</v>
+      </c>
+      <c r="I391" s="3">
+        <f t="shared" si="47"/>
+        <v>1.2419293528819231</v>
+      </c>
+    </row>
+    <row r="392" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A392" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B392" s="3">
+        <v>1504</v>
+      </c>
+      <c r="C392" s="3">
+        <v>3572.56</v>
+      </c>
+      <c r="D392" s="3">
+        <f>C392*(1/B392)^(2/3)</f>
+        <v>27.215374020088067</v>
+      </c>
+      <c r="E392" s="25" t="s">
+        <v>661</v>
+      </c>
+      <c r="F392" s="25" t="s">
+        <v>679</v>
+      </c>
+      <c r="G392" s="3">
+        <f t="shared" si="48"/>
+        <v>7.3158835045097854</v>
+      </c>
+      <c r="H392" s="3">
+        <f t="shared" si="49"/>
+        <v>8.1810377046245009</v>
+      </c>
+      <c r="I392" s="3">
+        <f t="shared" si="47"/>
+        <v>0.34191033843272634</v>
+      </c>
+    </row>
+    <row r="393" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A393" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="B393" s="3">
+        <v>350</v>
+      </c>
+      <c r="C393" s="3">
+        <v>1936.8200859999999</v>
+      </c>
+      <c r="D393" s="3">
+        <f>C393*(1/B393)^(2/3)</f>
+        <v>38.998142103730338</v>
+      </c>
+      <c r="E393" s="25" t="s">
+        <v>661</v>
+      </c>
+      <c r="F393" s="25" t="s">
+        <v>678</v>
+      </c>
+      <c r="G393" s="3">
+        <f t="shared" si="48"/>
+        <v>5.857933154483459</v>
+      </c>
+      <c r="H393" s="3">
+        <f t="shared" si="49"/>
+        <v>7.5688027762846541</v>
+      </c>
+      <c r="I393" s="3">
+        <f t="shared" si="47"/>
+        <v>0.51179380527576179</v>
+      </c>
+    </row>
+    <row r="394" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A394" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B394" s="3">
+        <v>12.14</v>
+      </c>
+      <c r="C394" s="3">
+        <v>288.69608849999997</v>
+      </c>
+      <c r="D394" s="3">
+        <f>C394*(1/B394)^(2/3)</f>
+        <v>54.654816673444103</v>
+      </c>
+      <c r="E394" s="25" t="s">
+        <v>661</v>
+      </c>
+      <c r="F394" s="25" t="s">
+        <v>650</v>
+      </c>
+      <c r="G394" s="3">
+        <f t="shared" si="48"/>
+        <v>2.4965057856313524</v>
+      </c>
+      <c r="H394" s="3">
+        <f t="shared" si="49"/>
+        <v>5.6653745379106697</v>
+      </c>
+      <c r="I394" s="3">
+        <f t="shared" si="47"/>
+        <v>0.79319087030179458</v>
+      </c>
+    </row>
+    <row r="395" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A395" s="2" t="s">
+        <v>657</v>
+      </c>
+      <c r="B395" s="3">
+        <v>13.0528220298457</v>
+      </c>
+      <c r="C395" s="3">
+        <v>392.93424750000003</v>
+      </c>
+      <c r="D395" s="3">
+        <f>C395*(1/B395)^(2/3)</f>
+        <v>70.878895024061563</v>
+      </c>
+      <c r="E395" s="25" t="s">
+        <v>661</v>
+      </c>
+      <c r="F395" s="25" t="s">
+        <v>650</v>
+      </c>
+      <c r="G395" s="3">
+        <f t="shared" si="48"/>
+        <v>2.5690043578883373</v>
+      </c>
+      <c r="H395" s="3">
+        <f t="shared" si="49"/>
+        <v>5.9736422887112175</v>
+      </c>
+      <c r="I395" s="3">
+        <f t="shared" si="47"/>
+        <v>1.0264167496369121</v>
+      </c>
+    </row>
+    <row r="396" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A396" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="B396" s="3">
+        <v>2700</v>
+      </c>
+      <c r="C396" s="3">
+        <v>16206.266589999999</v>
+      </c>
+      <c r="D396" s="3">
+        <f>C396*(1/B396)^(2/3)</f>
+        <v>83.580917820773152</v>
+      </c>
+      <c r="E396" s="25" t="s">
+        <v>661</v>
+      </c>
+      <c r="F396" s="25" t="s">
+        <v>678</v>
+      </c>
+      <c r="G396" s="3">
+        <f t="shared" si="48"/>
+        <v>7.90100705199242</v>
+      </c>
+      <c r="H396" s="3">
+        <f t="shared" si="49"/>
+        <v>9.6931532729655867</v>
+      </c>
+      <c r="I396" s="3">
+        <f t="shared" si="47"/>
+        <v>1.0318071305047645</v>
+      </c>
+    </row>
+    <row r="397" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A397" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="B397" s="3">
+        <v>2300</v>
+      </c>
+      <c r="C397" s="3">
+        <v>16641.29681</v>
+      </c>
+      <c r="D397" s="3">
+        <f>C397*(1/B397)^(2/3)</f>
+        <v>95.50701592966432</v>
+      </c>
+      <c r="E397" s="25" t="s">
+        <v>661</v>
+      </c>
+      <c r="F397" s="25" t="s">
+        <v>677</v>
+      </c>
+      <c r="G397" s="3">
+        <f t="shared" si="48"/>
+        <v>7.7406644019172415</v>
+      </c>
+      <c r="H397" s="3">
+        <f t="shared" si="49"/>
+        <v>9.7196426446318274</v>
+      </c>
+      <c r="I397" s="3">
+        <f t="shared" si="47"/>
+        <v>1.1847073976188882</v>
+      </c>
+    </row>
+    <row r="398" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A398" s="2" t="s">
+        <v>659</v>
+      </c>
+      <c r="B398" s="3">
+        <v>1013</v>
+      </c>
+      <c r="C398" s="3">
+        <v>13816.80804</v>
+      </c>
+      <c r="D398" s="3">
+        <f>C398*(1/B398)^(2/3)</f>
+        <v>136.98344801185283</v>
+      </c>
+      <c r="E398" s="25" t="s">
+        <v>661</v>
+      </c>
+      <c r="F398" s="25" t="s">
+        <v>676</v>
+      </c>
+      <c r="G398" s="3">
+        <f t="shared" si="48"/>
+        <v>6.9206715042486833</v>
+      </c>
+      <c r="H398" s="3">
+        <f t="shared" si="49"/>
+        <v>9.5336411039298348</v>
+      </c>
+      <c r="I398" s="3">
+        <f t="shared" si="47"/>
+        <v>1.7414208040342054</v>
+      </c>
+    </row>
+    <row r="399" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A399" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="B399" s="3">
+        <v>6.3140280461379197</v>
+      </c>
+      <c r="C399" s="3">
+        <v>249.65756540000001</v>
+      </c>
+      <c r="D399" s="3">
+        <f>C399*(1/B399)^(2/3)</f>
+        <v>73.081433915868459</v>
+      </c>
+      <c r="E399" s="25" t="s">
+        <v>661</v>
+      </c>
+      <c r="F399" s="25" t="s">
+        <v>650</v>
+      </c>
+      <c r="G399" s="3">
+        <f t="shared" si="48"/>
+        <v>1.8427738320229761</v>
+      </c>
+      <c r="H399" s="3">
+        <f t="shared" si="49"/>
+        <v>5.5200902405130963</v>
+      </c>
+      <c r="I399" s="3">
+        <f t="shared" si="47"/>
+        <v>1.0815703243524957</v>
+      </c>
+    </row>
+    <row r="400" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A400" s="2" t="s">
+        <v>664</v>
+      </c>
+      <c r="B400" s="3">
+        <v>6177.04</v>
+      </c>
+      <c r="C400" s="3">
+        <v>16984</v>
+      </c>
+      <c r="D400" s="3">
+        <f>C400*(1/B400)^(2/3)</f>
+        <v>50.44905536840853</v>
+      </c>
+      <c r="E400" s="26" t="s">
+        <v>237</v>
+      </c>
+      <c r="F400" s="26" t="s">
+        <v>680</v>
+      </c>
+      <c r="G400" s="3">
+        <f t="shared" ref="G400:G405" si="50">LN(B400)</f>
+        <v>8.7285944713103536</v>
+      </c>
+      <c r="H400" s="3">
+        <f t="shared" ref="H400:H406" si="51">LN(C400)</f>
+        <v>9.7400270033830925</v>
+      </c>
+      <c r="I400" s="3">
+        <f t="shared" si="47"/>
+        <v>0.60755540557612009</v>
+      </c>
+    </row>
+    <row r="401" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A401" s="2" t="s">
+        <v>665</v>
+      </c>
+      <c r="B401" s="3">
+        <f>POWER(10,2.754*LOG(350)-0.683)/1000</f>
+        <v>2105.539504495147</v>
+      </c>
+      <c r="C401" s="3">
+        <v>3416.3204929243898</v>
+      </c>
+      <c r="D401" s="3">
+        <f>C401*(1/B401)^(2/3)</f>
+        <v>20.796153290643581</v>
+      </c>
+      <c r="E401" s="26" t="s">
+        <v>237</v>
+      </c>
+      <c r="F401" s="10" t="s">
+        <v>692</v>
+      </c>
+      <c r="G401" s="3">
+        <f t="shared" si="50"/>
+        <v>7.6523270099503797</v>
+      </c>
+      <c r="H401" s="3">
+        <f t="shared" si="51"/>
+        <v>8.1363193716212319</v>
+      </c>
+      <c r="I401" s="3">
+        <f t="shared" si="47"/>
+        <v>0.2586468597552094</v>
+      </c>
+    </row>
+    <row r="402" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A402" s="2" t="s">
+        <v>666</v>
+      </c>
+      <c r="B402" s="3">
+        <v>6325</v>
+      </c>
+      <c r="C402" s="3">
+        <v>25449.1975520052</v>
+      </c>
+      <c r="D402" s="3">
+        <f>C402*(1/B402)^(2/3)</f>
+        <v>74.410417240525206</v>
+      </c>
+      <c r="E402" s="26" t="s">
+        <v>237</v>
+      </c>
+      <c r="F402" s="10" t="s">
+        <v>687</v>
+      </c>
+      <c r="G402" s="3">
+        <f t="shared" si="50"/>
+        <v>8.7522653135957214</v>
+      </c>
+      <c r="H402" s="3">
+        <f t="shared" si="51"/>
+        <v>10.1444394911085</v>
+      </c>
+      <c r="I402" s="3">
+        <f t="shared" si="47"/>
+        <v>0.89548614774219459</v>
+      </c>
+    </row>
+    <row r="403" spans="1:9" s="26" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A403" s="2" t="s">
+        <v>651</v>
+      </c>
+      <c r="B403" s="3">
+        <v>1743</v>
+      </c>
+      <c r="C403" s="3">
+        <v>7171.6109809273803</v>
+      </c>
+      <c r="D403" s="3">
+        <f>C403*(1/B403)^(2/3)</f>
+        <v>49.516711972852427</v>
+      </c>
+      <c r="E403" s="26" t="s">
+        <v>237</v>
+      </c>
+      <c r="F403" s="26" t="s">
+        <v>681</v>
+      </c>
+      <c r="G403" s="3">
+        <f t="shared" si="50"/>
+        <v>7.4633630455200208</v>
+      </c>
+      <c r="H403" s="3">
+        <f t="shared" si="51"/>
+        <v>8.8778855918885107</v>
+      </c>
+      <c r="I403" s="3">
+        <f t="shared" si="47"/>
+        <v>0.61934481752458748</v>
+      </c>
+    </row>
+    <row r="404" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A404" s="2" t="s">
+        <v>667</v>
+      </c>
+      <c r="B404" s="3">
+        <v>524</v>
+      </c>
+      <c r="C404" s="3">
+        <v>5998.3563019004296</v>
+      </c>
+      <c r="D404" s="3">
+        <f>C404*(1/B404)^(2/3)</f>
+        <v>92.28789379743678</v>
+      </c>
+      <c r="E404" s="26" t="s">
+        <v>237</v>
+      </c>
+      <c r="F404" s="26" t="s">
+        <v>683</v>
+      </c>
+      <c r="G404" s="3">
+        <f t="shared" si="50"/>
+        <v>6.261491684321042</v>
+      </c>
+      <c r="H404" s="3">
+        <f t="shared" si="51"/>
+        <v>8.6992407609958615</v>
+      </c>
+      <c r="I404" s="3">
+        <f t="shared" si="47"/>
+        <v>1.1966017371342328</v>
+      </c>
+    </row>
+    <row r="405" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A405" s="2" t="s">
+        <v>668</v>
+      </c>
+      <c r="B405" s="3">
+        <v>42</v>
+      </c>
+      <c r="C405" s="3">
+        <v>706.023203879584</v>
+      </c>
+      <c r="D405" s="3">
+        <f>C405*(1/B405)^(2/3)</f>
+        <v>58.432273061750777</v>
+      </c>
+      <c r="E405" s="26" t="s">
+        <v>237</v>
+      </c>
+      <c r="F405" s="26" t="s">
+        <v>684</v>
+      </c>
+      <c r="G405" s="3">
+        <f t="shared" si="50"/>
+        <v>3.7376696182833684</v>
+      </c>
+      <c r="H405" s="3">
+        <f t="shared" si="51"/>
+        <v>6.559648103638108</v>
+      </c>
+      <c r="I405" s="3">
+        <f t="shared" si="47"/>
+        <v>0.81708467145677222</v>
+      </c>
+    </row>
+    <row r="406" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A406" s="2" t="s">
+        <v>671</v>
+      </c>
+      <c r="B406" s="3">
+        <v>7390</v>
+      </c>
+      <c r="C406" s="3">
+        <v>11935.6168365434</v>
+      </c>
+      <c r="D406" s="3">
+        <f>C406*(1/B406)^(2/3)</f>
+        <v>31.459265318184478</v>
+      </c>
+      <c r="E406" s="26" t="s">
+        <v>237</v>
+      </c>
+      <c r="F406" s="26" t="s">
+        <v>685</v>
+      </c>
+      <c r="G406" s="3">
+        <f t="shared" ref="G406:G410" si="52">LN(B406)</f>
+        <v>8.9078830139422482</v>
+      </c>
+      <c r="H406" s="3">
+        <f t="shared" ref="H406:H410" si="53">LN(C406)</f>
+        <v>9.3872822204322492</v>
+      </c>
+      <c r="I406" s="3">
+        <f t="shared" si="47"/>
+        <v>0.37683453500109182</v>
+      </c>
+    </row>
+    <row r="407" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A407" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="B407" s="3">
+        <f>(280/230)*(280/230)*(280/230)*15</f>
+        <v>27.063368126900638</v>
+      </c>
+      <c r="C407" s="3">
+        <v>304.38665913735002</v>
+      </c>
+      <c r="D407" s="3">
+        <f>C407*(1/B407)^(2/3)</f>
+        <v>33.76792572973492</v>
+      </c>
+      <c r="E407" s="26" t="s">
+        <v>237</v>
+      </c>
+      <c r="F407" s="26" t="s">
+        <v>688</v>
+      </c>
+      <c r="G407" s="3">
+        <f t="shared" si="52"/>
+        <v>3.2981810838403729</v>
+      </c>
+      <c r="H407" s="3">
+        <f t="shared" si="53"/>
+        <v>5.7182987982772753</v>
+      </c>
+      <c r="I407" s="3">
+        <f t="shared" si="47"/>
+        <v>0.47844493899746898</v>
+      </c>
+    </row>
+    <row r="408" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A408" s="2" t="s">
+        <v>673</v>
+      </c>
+      <c r="B408" s="3">
+        <v>1330</v>
+      </c>
+      <c r="C408" s="3">
+        <v>6312.2812749765799</v>
+      </c>
+      <c r="D408" s="3">
+        <f>C408*(1/B408)^(2/3)</f>
+        <v>52.193759746907674</v>
+      </c>
+      <c r="E408" s="26" t="s">
+        <v>237</v>
+      </c>
+      <c r="F408" s="26" t="s">
+        <v>686</v>
+      </c>
+      <c r="G408" s="3">
+        <f t="shared" si="52"/>
+        <v>7.1929342212157996</v>
+      </c>
+      <c r="H408" s="3">
+        <f t="shared" si="53"/>
+        <v>8.750252423474647</v>
+      </c>
+      <c r="I408" s="3">
+        <f t="shared" si="47"/>
+        <v>0.65813476735142062</v>
+      </c>
+    </row>
+    <row r="409" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A409" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="B409" s="3">
+        <v>475</v>
+      </c>
+      <c r="C409" s="3">
+        <v>3872.3915755647599</v>
+      </c>
+      <c r="D409" s="3">
+        <f>C409*(1/B409)^(2/3)</f>
+        <v>63.608749860925712</v>
+      </c>
+      <c r="E409" s="26" t="s">
+        <v>237</v>
+      </c>
+      <c r="F409" s="26" t="s">
+        <v>689</v>
+      </c>
+      <c r="G409" s="3">
+        <f t="shared" si="52"/>
+        <v>6.1633148040346413</v>
+      </c>
+      <c r="H409" s="3">
+        <f t="shared" si="53"/>
+        <v>8.2616275733360514</v>
+      </c>
+      <c r="I409" s="3">
+        <f t="shared" si="47"/>
+        <v>0.82717622336571062</v>
+      </c>
+    </row>
+    <row r="410" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A410" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="B410" s="3">
+        <v>440</v>
+      </c>
+      <c r="C410" s="10">
+        <v>242.50025470955799</v>
+      </c>
+      <c r="D410" s="3">
+        <f t="shared" ref="D406:D410" si="54">C410*(1/B410)^(2/3)</f>
+        <v>4.1918951835589917</v>
+      </c>
+      <c r="E410" s="26" t="s">
+        <v>237</v>
+      </c>
+      <c r="F410" s="26" t="s">
+        <v>690</v>
+      </c>
+      <c r="G410" s="3">
+        <f t="shared" si="52"/>
+        <v>6.0867747269123065</v>
+      </c>
+      <c r="H410" s="3">
+        <f t="shared" si="53"/>
+        <v>5.4910027607256788</v>
+      </c>
+      <c r="I410" s="3">
+        <f>C410/EXP(0.6966*LN(B410)+4.158)</f>
+        <v>5.4636970278415457E-2</v>
+      </c>
+    </row>
+    <row r="411" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E411" s="26"/>
+      <c r="F411" s="26"/>
+    </row>
+    <row r="412" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E412" s="26"/>
+      <c r="F412" s="26"/>
+    </row>
+    <row r="413" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E413" s="26"/>
+      <c r="F413" s="26"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A266:H266"/>
     <mergeCell ref="A312:H312"/>
     <mergeCell ref="A337:H337"/>
+    <mergeCell ref="A381:H381"/>
     <mergeCell ref="A341:H341"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A39:H39"/>
@@ -33464,6 +35018,7 @@
     <mergeCell ref="A180:H180"/>
     <mergeCell ref="A262:H262"/>
   </mergeCells>
+  <phoneticPr fontId="11" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="F124" r:id="rId1" xr:uid="{0ED39283-3411-4AD9-AB09-B91C2DF53A20}"/>
   </hyperlinks>
@@ -48055,12 +49610,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="29" t="s">
         <v>581</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
     </row>
     <row r="2" spans="1:4" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
@@ -54804,14 +56359,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="27" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
     </row>
     <row r="2" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
@@ -56042,17 +57597,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="27" t="s">
         <v>391</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
@@ -56859,14 +58414,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="27" t="s">
         <v>224</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">

</xml_diff>